<commit_message>
Re-run matching with updated cashflow file (9,290 rows)
Updated cashflow source file to new version with more entries.
Match count improved from 389 to 593 out of 916 transactions.

https://claude.ai/code/session_01XeMrDPbEZpTmVXhm7fguJk
</commit_message>
<xml_diff>
--- a/입출금내역_4월_프로젝트매칭.xlsx
+++ b/입출금내역_4월_프로젝트매칭.xlsx
@@ -1021,7 +1021,11 @@
         </is>
       </c>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>I250416(야적장 갠트리크레인 설치공사)-C</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1129,7 +1133,7 @@
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>E260001(경비-임대)-E</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1186,11 @@
         </is>
       </c>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1237,7 +1245,11 @@
           <t>하자</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>L251203(위례푸른초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1292,7 +1304,11 @@
           <t>하자</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>L251202(청주성신학교)-A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1343,7 +1359,11 @@
         </is>
       </c>
       <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1396,7 +1416,7 @@
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t xml:space="preserve">A260102(군산공장 천정크레인)-E </t>
         </is>
       </c>
     </row>
@@ -1449,7 +1469,11 @@
         </is>
       </c>
       <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>L211101(홍성 한울초)-D</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1500,7 +1524,11 @@
         </is>
       </c>
       <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>L240404(순천공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1553,7 +1581,7 @@
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4현장실)-C</t>
+          <t>L251003(연무마이스터고)-A</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1685,11 @@
         </is>
       </c>
       <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>L251003(연무마이스터고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1708,7 +1740,11 @@
         </is>
       </c>
       <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>E260002(경비-김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1759,7 +1795,11 @@
         </is>
       </c>
       <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>D250506(OSC 고도화 기술개발사업-PC공동주택)-E</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1810,7 +1850,11 @@
         </is>
       </c>
       <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>S251102(BC양구 간부숙소)-M</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1861,7 +1905,11 @@
         </is>
       </c>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>S251102(BC양구 간부숙소)-M</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1912,7 +1960,11 @@
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>E260001(경비-임대)-E</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1963,7 +2015,11 @@
         </is>
       </c>
       <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>E260001(경비-임대)-E</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2615,7 +2671,11 @@
         </is>
       </c>
       <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2717,7 +2777,11 @@
         </is>
       </c>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2770,7 +2834,7 @@
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>C240801(의왕초평A-4BL)-M</t>
         </is>
       </c>
     </row>
@@ -2988,7 +3052,11 @@
         </is>
       </c>
       <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>L211201(대전 버드내중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3094,7 +3162,11 @@
         </is>
       </c>
       <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3145,7 +3217,11 @@
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3196,7 +3272,11 @@
         </is>
       </c>
       <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>L230805(태백 세연중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -6254,7 +6334,11 @@
         </is>
       </c>
       <c r="N110" t="inlineStr"/>
-      <c r="O110" t="inlineStr"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -6305,7 +6389,11 @@
         </is>
       </c>
       <c r="N111" t="inlineStr"/>
-      <c r="O111" t="inlineStr"/>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -6356,7 +6444,11 @@
         </is>
       </c>
       <c r="N112" t="inlineStr"/>
-      <c r="O112" t="inlineStr"/>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -6792,7 +6884,11 @@
         </is>
       </c>
       <c r="N120" t="inlineStr"/>
-      <c r="O120" t="inlineStr"/>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>L230805(태백 세연중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -7008,7 +7104,11 @@
         </is>
       </c>
       <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr"/>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -7059,7 +7159,11 @@
         </is>
       </c>
       <c r="N125" t="inlineStr"/>
-      <c r="O125" t="inlineStr"/>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -7167,7 +7271,7 @@
       <c r="N127" t="inlineStr"/>
       <c r="O127" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>C240801(의왕초평A-4BL)-M</t>
         </is>
       </c>
     </row>
@@ -9826,7 +9930,7 @@
       <c r="N176" t="inlineStr"/>
       <c r="O176" t="inlineStr">
         <is>
-          <t>L250418(대구 경상여고)-A</t>
+          <t>L251202(청주성신학교)-A</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9983,11 @@
         </is>
       </c>
       <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>L250420(동해 북평초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -9930,7 +10038,11 @@
         </is>
       </c>
       <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr"/>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>L250302(진천 백곡초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -9981,7 +10093,11 @@
         </is>
       </c>
       <c r="N179" t="inlineStr"/>
-      <c r="O179" t="inlineStr"/>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -10032,7 +10148,11 @@
         </is>
       </c>
       <c r="N180" t="inlineStr"/>
-      <c r="O180" t="inlineStr"/>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -10083,7 +10203,11 @@
         </is>
       </c>
       <c r="N181" t="inlineStr"/>
-      <c r="O181" t="inlineStr"/>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>L251202(청주성신학교)-A</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -10134,7 +10258,11 @@
         </is>
       </c>
       <c r="N182" t="inlineStr"/>
-      <c r="O182" t="inlineStr"/>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>L250420(동해 북평초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -10185,7 +10313,11 @@
         </is>
       </c>
       <c r="N183" t="inlineStr"/>
-      <c r="O183" t="inlineStr"/>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -10236,7 +10368,11 @@
         </is>
       </c>
       <c r="N184" t="inlineStr"/>
-      <c r="O184" t="inlineStr"/>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>L251005(홍성공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -10287,7 +10423,11 @@
         </is>
       </c>
       <c r="N185" t="inlineStr"/>
-      <c r="O185" t="inlineStr"/>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -10338,7 +10478,11 @@
         </is>
       </c>
       <c r="N186" t="inlineStr"/>
-      <c r="O186" t="inlineStr"/>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -10389,7 +10533,11 @@
         </is>
       </c>
       <c r="N187" t="inlineStr"/>
-      <c r="O187" t="inlineStr"/>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -10440,7 +10588,11 @@
         </is>
       </c>
       <c r="N188" t="inlineStr"/>
-      <c r="O188" t="inlineStr"/>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -10491,7 +10643,11 @@
         </is>
       </c>
       <c r="N189" t="inlineStr"/>
-      <c r="O189" t="inlineStr"/>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>E250003(경비-기타)-E</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -10593,7 +10749,11 @@
         </is>
       </c>
       <c r="N191" t="inlineStr"/>
-      <c r="O191" t="inlineStr"/>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평 A-4BL TF)-P</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -10644,7 +10804,11 @@
         </is>
       </c>
       <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr"/>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -10695,7 +10859,11 @@
         </is>
       </c>
       <c r="N193" t="inlineStr"/>
-      <c r="O193" t="inlineStr"/>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -10797,7 +10965,11 @@
         </is>
       </c>
       <c r="N195" t="inlineStr"/>
-      <c r="O195" t="inlineStr"/>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>L260203(강원 양양고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -11335,7 +11507,11 @@
         </is>
       </c>
       <c r="N205" t="inlineStr"/>
-      <c r="O205" t="inlineStr"/>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -12567,7 +12743,11 @@
         </is>
       </c>
       <c r="N229" t="inlineStr"/>
-      <c r="O229" t="inlineStr"/>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>L230205(충남 태안중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -12620,7 +12800,7 @@
       <c r="N230" t="inlineStr"/>
       <c r="O230" t="inlineStr">
         <is>
-          <t>L250418(대구 경상여고)-A</t>
+          <t>L251005(홍성공고)-A</t>
         </is>
       </c>
     </row>
@@ -12673,7 +12853,11 @@
         </is>
       </c>
       <c r="N231" t="inlineStr"/>
-      <c r="O231" t="inlineStr"/>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>L250804(김해 대중초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -12724,7 +12908,11 @@
         </is>
       </c>
       <c r="N232" t="inlineStr"/>
-      <c r="O232" t="inlineStr"/>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>L250804(김해 대중초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -12775,7 +12963,11 @@
         </is>
       </c>
       <c r="N233" t="inlineStr"/>
-      <c r="O233" t="inlineStr"/>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -12826,7 +13018,11 @@
         </is>
       </c>
       <c r="N234" t="inlineStr"/>
-      <c r="O234" t="inlineStr"/>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>L251005(홍성공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -12877,7 +13073,11 @@
         </is>
       </c>
       <c r="N235" t="inlineStr"/>
-      <c r="O235" t="inlineStr"/>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>M251101(BS3-목업)-M</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -12983,7 +13183,11 @@
         </is>
       </c>
       <c r="N237" t="inlineStr"/>
-      <c r="O237" t="inlineStr"/>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>M251101(BS3-목업)-M</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -13462,7 +13666,11 @@
         </is>
       </c>
       <c r="N246" t="inlineStr"/>
-      <c r="O246" t="inlineStr"/>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>D241207(프리배브 UBR 욕실개발)-E</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -13568,7 +13776,11 @@
         </is>
       </c>
       <c r="N248" t="inlineStr"/>
-      <c r="O248" t="inlineStr"/>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>D250801(전북 혁신성장 R&amp;D+)-E</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -13621,7 +13833,7 @@
       <c r="N249" t="inlineStr"/>
       <c r="O249" t="inlineStr">
         <is>
-          <t>D250506(OSC 고도화 기술개발사업-PC공동주택)-E</t>
+          <t>M250902(BS3-25-A)-M</t>
         </is>
       </c>
     </row>
@@ -13674,7 +13886,11 @@
         </is>
       </c>
       <c r="N250" t="inlineStr"/>
-      <c r="O250" t="inlineStr"/>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>E250003(경비-기타)-E</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -13725,7 +13941,11 @@
         </is>
       </c>
       <c r="N251" t="inlineStr"/>
-      <c r="O251" t="inlineStr"/>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -13776,7 +13996,11 @@
         </is>
       </c>
       <c r="N252" t="inlineStr"/>
-      <c r="O252" t="inlineStr"/>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -13827,7 +14051,11 @@
         </is>
       </c>
       <c r="N253" t="inlineStr"/>
-      <c r="O253" t="inlineStr"/>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -13878,7 +14106,11 @@
         </is>
       </c>
       <c r="N254" t="inlineStr"/>
-      <c r="O254" t="inlineStr"/>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -13929,7 +14161,11 @@
         </is>
       </c>
       <c r="N255" t="inlineStr"/>
-      <c r="O255" t="inlineStr"/>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -13982,7 +14218,7 @@
       <c r="N256" t="inlineStr"/>
       <c r="O256" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>C240801(의왕초평A-4BL)-M</t>
         </is>
       </c>
     </row>
@@ -14035,7 +14271,11 @@
         </is>
       </c>
       <c r="N257" t="inlineStr"/>
-      <c r="O257" t="inlineStr"/>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -14086,7 +14326,11 @@
         </is>
       </c>
       <c r="N258" t="inlineStr"/>
-      <c r="O258" t="inlineStr"/>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -14137,7 +14381,11 @@
         </is>
       </c>
       <c r="N259" t="inlineStr"/>
-      <c r="O259" t="inlineStr"/>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -14188,7 +14436,11 @@
         </is>
       </c>
       <c r="N260" t="inlineStr"/>
-      <c r="O260" t="inlineStr"/>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>M250902(BS3-25-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -14239,7 +14491,11 @@
         </is>
       </c>
       <c r="N261" t="inlineStr"/>
-      <c r="O261" t="inlineStr"/>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -14465,7 +14721,7 @@
       <c r="N265" t="inlineStr"/>
       <c r="O265" t="inlineStr">
         <is>
-          <t>D250506(OSC 고도화 기술개발사업-PC공동주택)-E</t>
+          <t>M250902(BS3-25-A)-M</t>
         </is>
       </c>
     </row>
@@ -15425,7 +15681,11 @@
         </is>
       </c>
       <c r="N283" t="inlineStr"/>
-      <c r="O283" t="inlineStr"/>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -15994,7 +16254,11 @@
         </is>
       </c>
       <c r="N294" t="inlineStr"/>
-      <c r="O294" t="inlineStr"/>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>C240801(BH의왕초평A-4BL)-A</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -16045,7 +16309,11 @@
         </is>
       </c>
       <c r="N295" t="inlineStr"/>
-      <c r="O295" t="inlineStr"/>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>C240801(BH의왕초평A-4BL)-A</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -16573,7 +16841,7 @@
       <c r="N305" t="inlineStr"/>
       <c r="O305" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4BL)-M</t>
+          <t>C240801(의왕초평A-4현장실)-C</t>
         </is>
       </c>
     </row>
@@ -16626,7 +16894,11 @@
         </is>
       </c>
       <c r="N306" t="inlineStr"/>
-      <c r="O306" t="inlineStr"/>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -19765,7 +20037,11 @@
         </is>
       </c>
       <c r="N367" t="inlineStr"/>
-      <c r="O367" t="inlineStr"/>
+      <c r="O367" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -19816,7 +20092,11 @@
         </is>
       </c>
       <c r="N368" t="inlineStr"/>
-      <c r="O368" t="inlineStr"/>
+      <c r="O368" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -20895,7 +21175,11 @@
         </is>
       </c>
       <c r="N389" t="inlineStr"/>
-      <c r="O389" t="inlineStr"/>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -21315,7 +21599,11 @@
         </is>
       </c>
       <c r="N397" t="inlineStr"/>
-      <c r="O397" t="inlineStr"/>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="n">
@@ -21366,7 +21654,11 @@
         </is>
       </c>
       <c r="N398" t="inlineStr"/>
-      <c r="O398" t="inlineStr"/>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="n">
@@ -21417,7 +21709,11 @@
         </is>
       </c>
       <c r="N399" t="inlineStr"/>
-      <c r="O399" t="inlineStr"/>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>L240703(서산 음암중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -21908,7 +22204,11 @@
         </is>
       </c>
       <c r="N408" t="inlineStr"/>
-      <c r="O408" t="inlineStr"/>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="n">
@@ -22014,7 +22314,11 @@
         </is>
       </c>
       <c r="N410" t="inlineStr"/>
-      <c r="O410" t="inlineStr"/>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="n">
@@ -22065,7 +22369,11 @@
         </is>
       </c>
       <c r="N411" t="inlineStr"/>
-      <c r="O411" t="inlineStr"/>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="n">
@@ -22116,7 +22424,11 @@
         </is>
       </c>
       <c r="N412" t="inlineStr"/>
-      <c r="O412" t="inlineStr"/>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -22458,7 +22770,11 @@
         </is>
       </c>
       <c r="N418" t="inlineStr"/>
-      <c r="O418" t="inlineStr"/>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="n">
@@ -22619,7 +22935,11 @@
         </is>
       </c>
       <c r="N421" t="inlineStr"/>
-      <c r="O421" t="inlineStr"/>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
@@ -23726,7 +24046,11 @@
         </is>
       </c>
       <c r="N442" t="inlineStr"/>
-      <c r="O442" t="inlineStr"/>
+      <c r="O442" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" t="n">
@@ -23934,7 +24258,11 @@
         </is>
       </c>
       <c r="N446" t="inlineStr"/>
-      <c r="O446" t="inlineStr"/>
+      <c r="O446" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평 A-4BL TF)-P</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" t="n">
@@ -23985,7 +24313,11 @@
         </is>
       </c>
       <c r="N447" t="inlineStr"/>
-      <c r="O447" t="inlineStr"/>
+      <c r="O447" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평 A-4BL TF)-P</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" t="n">
@@ -24036,7 +24368,11 @@
         </is>
       </c>
       <c r="N448" t="inlineStr"/>
-      <c r="O448" t="inlineStr"/>
+      <c r="O448" t="inlineStr">
+        <is>
+          <t>C250704(소규모주택[완도,고흥])-P</t>
+        </is>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="n">
@@ -24087,7 +24423,11 @@
         </is>
       </c>
       <c r="N449" t="inlineStr"/>
-      <c r="O449" t="inlineStr"/>
+      <c r="O449" t="inlineStr">
+        <is>
+          <t>C250704(소규모주택[완도,고흥])-P</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" t="n">
@@ -24138,7 +24478,11 @@
         </is>
       </c>
       <c r="N450" t="inlineStr"/>
-      <c r="O450" t="inlineStr"/>
+      <c r="O450" t="inlineStr">
+        <is>
+          <t>C250704(소규모주택[완도,고흥])-P</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="n">
@@ -24189,7 +24533,11 @@
         </is>
       </c>
       <c r="N451" t="inlineStr"/>
-      <c r="O451" t="inlineStr"/>
+      <c r="O451" t="inlineStr">
+        <is>
+          <t>L260201(대전 유성여고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" t="n">
@@ -24240,7 +24588,11 @@
         </is>
       </c>
       <c r="N452" t="inlineStr"/>
-      <c r="O452" t="inlineStr"/>
+      <c r="O452" t="inlineStr">
+        <is>
+          <t>L260202(서산여고 2차증축)-A</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" t="n">
@@ -24291,7 +24643,11 @@
         </is>
       </c>
       <c r="N453" t="inlineStr"/>
-      <c r="O453" t="inlineStr"/>
+      <c r="O453" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="n">
@@ -25917,7 +26273,11 @@
         </is>
       </c>
       <c r="N483" t="inlineStr"/>
-      <c r="O483" t="inlineStr"/>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>S250401(대구 군위중)-A</t>
+        </is>
+      </c>
     </row>
     <row r="484">
       <c r="A484" t="n">
@@ -26188,7 +26548,11 @@
         </is>
       </c>
       <c r="N488" t="inlineStr"/>
-      <c r="O488" t="inlineStr"/>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" t="n">
@@ -26294,7 +26658,11 @@
         </is>
       </c>
       <c r="N490" t="inlineStr"/>
-      <c r="O490" t="inlineStr"/>
+      <c r="O490" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="491">
       <c r="A491" t="n">
@@ -28260,7 +28628,11 @@
         </is>
       </c>
       <c r="N528" t="inlineStr"/>
-      <c r="O528" t="inlineStr"/>
+      <c r="O528" t="inlineStr">
+        <is>
+          <t>D221114(경상연구개발비)-E</t>
+        </is>
+      </c>
     </row>
     <row r="529">
       <c r="A529" t="n">
@@ -30573,7 +30945,7 @@
       <c r="N573" t="inlineStr"/>
       <c r="O573" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t xml:space="preserve">A260102(군산공장 천정크레인)-E </t>
         </is>
       </c>
     </row>
@@ -30630,7 +31002,11 @@
           <t>하자</t>
         </is>
       </c>
-      <c r="O574" t="inlineStr"/>
+      <c r="O574" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="575">
       <c r="A575" t="n">
@@ -30681,7 +31057,11 @@
         </is>
       </c>
       <c r="N575" t="inlineStr"/>
-      <c r="O575" t="inlineStr"/>
+      <c r="O575" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="576">
       <c r="A576" t="n">
@@ -30732,7 +31112,11 @@
         </is>
       </c>
       <c r="N576" t="inlineStr"/>
-      <c r="O576" t="inlineStr"/>
+      <c r="O576" t="inlineStr">
+        <is>
+          <t>L260201(대전 유성여고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" t="n">
@@ -30783,7 +31167,11 @@
         </is>
       </c>
       <c r="N577" t="inlineStr"/>
-      <c r="O577" t="inlineStr"/>
+      <c r="O577" t="inlineStr">
+        <is>
+          <t>M250902(BS3-25-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" t="n">
@@ -30885,7 +31273,11 @@
         </is>
       </c>
       <c r="N579" t="inlineStr"/>
-      <c r="O579" t="inlineStr"/>
+      <c r="O579" t="inlineStr">
+        <is>
+          <t>M250902(BS3-25-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="580">
       <c r="A580" t="n">
@@ -30936,7 +31328,11 @@
         </is>
       </c>
       <c r="N580" t="inlineStr"/>
-      <c r="O580" t="inlineStr"/>
+      <c r="O580" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="581">
       <c r="A581" t="n">
@@ -30987,7 +31383,11 @@
         </is>
       </c>
       <c r="N581" t="inlineStr"/>
-      <c r="O581" t="inlineStr"/>
+      <c r="O581" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="582">
       <c r="A582" t="n">
@@ -31040,7 +31440,7 @@
       <c r="N582" t="inlineStr"/>
       <c r="O582" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4BL)-M</t>
+          <t>E250002(경비-공장)-E</t>
         </is>
       </c>
     </row>
@@ -31368,7 +31768,11 @@
         </is>
       </c>
       <c r="N588" t="inlineStr"/>
-      <c r="O588" t="inlineStr"/>
+      <c r="O588" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="589">
       <c r="A589" t="n">
@@ -31474,7 +31878,11 @@
         </is>
       </c>
       <c r="N590" t="inlineStr"/>
-      <c r="O590" t="inlineStr"/>
+      <c r="O590" t="inlineStr">
+        <is>
+          <t>L251003(연무마이스터고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="591">
       <c r="A591" t="n">
@@ -31527,7 +31935,7 @@
       <c r="N591" t="inlineStr"/>
       <c r="O591" t="inlineStr">
         <is>
-          <t>M250902(BS3-25-A)-M</t>
+          <t>I260101(일체형지붕-강내초,부곡초,조례초,연동초,청산고)-E</t>
         </is>
       </c>
     </row>
@@ -31580,7 +31988,11 @@
         </is>
       </c>
       <c r="N592" t="inlineStr"/>
-      <c r="O592" t="inlineStr"/>
+      <c r="O592" t="inlineStr">
+        <is>
+          <t>I250416(배터리몰드 설치공사)-E</t>
+        </is>
+      </c>
     </row>
     <row r="593">
       <c r="A593" t="n">
@@ -31631,7 +32043,11 @@
         </is>
       </c>
       <c r="N593" t="inlineStr"/>
-      <c r="O593" t="inlineStr"/>
+      <c r="O593" t="inlineStr">
+        <is>
+          <t>L250804(김해 대중초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="594">
       <c r="A594" t="n">
@@ -31682,7 +32098,11 @@
         </is>
       </c>
       <c r="N594" t="inlineStr"/>
-      <c r="O594" t="inlineStr"/>
+      <c r="O594" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="595">
       <c r="A595" t="n">
@@ -31898,7 +32318,11 @@
         </is>
       </c>
       <c r="N598" t="inlineStr"/>
-      <c r="O598" t="inlineStr"/>
+      <c r="O598" t="inlineStr">
+        <is>
+          <t>L230208(충남 청양중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="599">
       <c r="A599" t="n">
@@ -32279,7 +32703,11 @@
         </is>
       </c>
       <c r="N605" t="inlineStr"/>
-      <c r="O605" t="inlineStr"/>
+      <c r="O605" t="inlineStr">
+        <is>
+          <t>M260204(BS3-26-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="606">
       <c r="A606" t="n">
@@ -32330,7 +32758,11 @@
         </is>
       </c>
       <c r="N606" t="inlineStr"/>
-      <c r="O606" t="inlineStr"/>
+      <c r="O606" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" t="n">
@@ -32432,7 +32864,11 @@
         </is>
       </c>
       <c r="N608" t="inlineStr"/>
-      <c r="O608" t="inlineStr"/>
+      <c r="O608" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="609">
       <c r="A609" t="n">
@@ -32483,7 +32919,11 @@
         </is>
       </c>
       <c r="N609" t="inlineStr"/>
-      <c r="O609" t="inlineStr"/>
+      <c r="O609" t="inlineStr">
+        <is>
+          <t>S250401(대구 군위중)-A</t>
+        </is>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="n">
@@ -32699,7 +33139,11 @@
         </is>
       </c>
       <c r="N613" t="inlineStr"/>
-      <c r="O613" t="inlineStr"/>
+      <c r="O613" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="614">
       <c r="A614" t="n">
@@ -32750,7 +33194,11 @@
         </is>
       </c>
       <c r="N614" t="inlineStr"/>
-      <c r="O614" t="inlineStr"/>
+      <c r="O614" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="615">
       <c r="A615" t="n">
@@ -32801,7 +33249,11 @@
         </is>
       </c>
       <c r="N615" t="inlineStr"/>
-      <c r="O615" t="inlineStr"/>
+      <c r="O615" t="inlineStr">
+        <is>
+          <t>A251201(김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="616">
       <c r="A616" t="n">
@@ -32854,7 +33306,7 @@
       <c r="N616" t="inlineStr"/>
       <c r="O616" t="inlineStr">
         <is>
-          <t>E260002(경비-김제공장)-E</t>
+          <t>A251201(김제공장)-E</t>
         </is>
       </c>
     </row>
@@ -32962,7 +33414,11 @@
         </is>
       </c>
       <c r="N618" t="inlineStr"/>
-      <c r="O618" t="inlineStr"/>
+      <c r="O618" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="619">
       <c r="A619" t="n">
@@ -33178,7 +33634,11 @@
         </is>
       </c>
       <c r="N622" t="inlineStr"/>
-      <c r="O622" t="inlineStr"/>
+      <c r="O622" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="623">
       <c r="A623" t="n">
@@ -33339,7 +33799,11 @@
         </is>
       </c>
       <c r="N625" t="inlineStr"/>
-      <c r="O625" t="inlineStr"/>
+      <c r="O625" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="626">
       <c r="A626" t="n">
@@ -33390,7 +33854,11 @@
         </is>
       </c>
       <c r="N626" t="inlineStr"/>
-      <c r="O626" t="inlineStr"/>
+      <c r="O626" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="n">
@@ -33441,7 +33909,11 @@
         </is>
       </c>
       <c r="N627" t="inlineStr"/>
-      <c r="O627" t="inlineStr"/>
+      <c r="O627" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="628">
       <c r="A628" t="n">
@@ -33492,7 +33964,11 @@
         </is>
       </c>
       <c r="N628" t="inlineStr"/>
-      <c r="O628" t="inlineStr"/>
+      <c r="O628" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="629">
       <c r="A629" t="n">
@@ -33543,7 +34019,11 @@
         </is>
       </c>
       <c r="N629" t="inlineStr"/>
-      <c r="O629" t="inlineStr"/>
+      <c r="O629" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="630">
       <c r="A630" t="n">
@@ -33594,7 +34074,11 @@
         </is>
       </c>
       <c r="N630" t="inlineStr"/>
-      <c r="O630" t="inlineStr"/>
+      <c r="O630" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="631">
       <c r="A631" t="n">
@@ -33645,7 +34129,11 @@
         </is>
       </c>
       <c r="N631" t="inlineStr"/>
-      <c r="O631" t="inlineStr"/>
+      <c r="O631" t="inlineStr">
+        <is>
+          <t>L260201(대전 유성여고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="632">
       <c r="A632" t="n">
@@ -33696,7 +34184,11 @@
         </is>
       </c>
       <c r="N632" t="inlineStr"/>
-      <c r="O632" t="inlineStr"/>
+      <c r="O632" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="633">
       <c r="A633" t="n">
@@ -33859,7 +34351,7 @@
       <c r="N635" t="inlineStr"/>
       <c r="O635" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4BL)-M</t>
+          <t>M260204(BS3-26-A)-M</t>
         </is>
       </c>
     </row>
@@ -33912,7 +34404,11 @@
         </is>
       </c>
       <c r="N636" t="inlineStr"/>
-      <c r="O636" t="inlineStr"/>
+      <c r="O636" t="inlineStr">
+        <is>
+          <t>I260103(대전 원신흥초)-E</t>
+        </is>
+      </c>
     </row>
     <row r="637">
       <c r="A637" t="n">
@@ -33963,7 +34459,11 @@
         </is>
       </c>
       <c r="N637" t="inlineStr"/>
-      <c r="O637" t="inlineStr"/>
+      <c r="O637" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4현장실)-C</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" t="n">
@@ -34014,7 +34514,11 @@
         </is>
       </c>
       <c r="N638" t="inlineStr"/>
-      <c r="O638" t="inlineStr"/>
+      <c r="O638" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" t="n">
@@ -34065,7 +34569,11 @@
         </is>
       </c>
       <c r="N639" t="inlineStr"/>
-      <c r="O639" t="inlineStr"/>
+      <c r="O639" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" t="n">
@@ -34116,7 +34624,11 @@
         </is>
       </c>
       <c r="N640" t="inlineStr"/>
-      <c r="O640" t="inlineStr"/>
+      <c r="O640" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="641">
       <c r="A641" t="n">
@@ -34167,7 +34679,11 @@
         </is>
       </c>
       <c r="N641" t="inlineStr"/>
-      <c r="O641" t="inlineStr"/>
+      <c r="O641" t="inlineStr">
+        <is>
+          <t>L251203(위례푸른초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="642">
       <c r="A642" t="n">
@@ -34218,7 +34734,11 @@
         </is>
       </c>
       <c r="N642" t="inlineStr"/>
-      <c r="O642" t="inlineStr"/>
+      <c r="O642" t="inlineStr">
+        <is>
+          <t>L251203(위례푸른초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" t="n">
@@ -34269,7 +34789,11 @@
         </is>
       </c>
       <c r="N643" t="inlineStr"/>
-      <c r="O643" t="inlineStr"/>
+      <c r="O643" t="inlineStr">
+        <is>
+          <t>S250401(대구 군위중)-A</t>
+        </is>
+      </c>
     </row>
     <row r="644">
       <c r="A644" t="n">
@@ -34320,7 +34844,11 @@
         </is>
       </c>
       <c r="N644" t="inlineStr"/>
-      <c r="O644" t="inlineStr"/>
+      <c r="O644" t="inlineStr">
+        <is>
+          <t>L230208(충남 청양중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" t="n">
@@ -34371,7 +34899,11 @@
         </is>
       </c>
       <c r="N645" t="inlineStr"/>
-      <c r="O645" t="inlineStr"/>
+      <c r="O645" t="inlineStr">
+        <is>
+          <t>L251005(홍성공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="646">
       <c r="A646" t="n">
@@ -34422,7 +34954,11 @@
         </is>
       </c>
       <c r="N646" t="inlineStr"/>
-      <c r="O646" t="inlineStr"/>
+      <c r="O646" t="inlineStr">
+        <is>
+          <t>L260202(서산여고 2차증축)-A</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" t="n">
@@ -34583,7 +35119,11 @@
         </is>
       </c>
       <c r="N649" t="inlineStr"/>
-      <c r="O649" t="inlineStr"/>
+      <c r="O649" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" t="n">
@@ -34634,7 +35174,11 @@
         </is>
       </c>
       <c r="N650" t="inlineStr"/>
-      <c r="O650" t="inlineStr"/>
+      <c r="O650" t="inlineStr">
+        <is>
+          <t>M260204(BS3-26-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="651">
       <c r="A651" t="n">
@@ -34685,7 +35229,11 @@
         </is>
       </c>
       <c r="N651" t="inlineStr"/>
-      <c r="O651" t="inlineStr"/>
+      <c r="O651" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" t="n">
@@ -34958,7 +35506,7 @@
       <c r="N656" t="inlineStr"/>
       <c r="O656" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4BL)-M</t>
+          <t>M260204(BS3-26-A)-M</t>
         </is>
       </c>
     </row>
@@ -35011,7 +35559,11 @@
         </is>
       </c>
       <c r="N657" t="inlineStr"/>
-      <c r="O657" t="inlineStr"/>
+      <c r="O657" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="658">
       <c r="A658" t="n">
@@ -35064,7 +35616,7 @@
       <c r="N658" t="inlineStr"/>
       <c r="O658" t="inlineStr">
         <is>
-          <t>D250801(전북 혁신성장 R&amp;D+)-E</t>
+          <t>D221114(경상연구개발비)-E</t>
         </is>
       </c>
     </row>
@@ -35119,7 +35671,7 @@
       <c r="N659" t="inlineStr"/>
       <c r="O659" t="inlineStr">
         <is>
-          <t>D250801(전북 혁신성장 R&amp;D+)-E</t>
+          <t>D221114(경상연구개발비)-E</t>
         </is>
       </c>
     </row>
@@ -35172,7 +35724,11 @@
         </is>
       </c>
       <c r="N660" t="inlineStr"/>
-      <c r="O660" t="inlineStr"/>
+      <c r="O660" t="inlineStr">
+        <is>
+          <t>C240801(BH의왕초평A-4BL)-A</t>
+        </is>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="n">
@@ -35223,7 +35779,11 @@
         </is>
       </c>
       <c r="N661" t="inlineStr"/>
-      <c r="O661" t="inlineStr"/>
+      <c r="O661" t="inlineStr">
+        <is>
+          <t>L260203(강원 양양고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="662">
       <c r="A662" t="n">
@@ -35276,7 +35836,7 @@
       <c r="N662" t="inlineStr"/>
       <c r="O662" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>L230805(태백 세연중)-D</t>
         </is>
       </c>
     </row>
@@ -35329,7 +35889,11 @@
         </is>
       </c>
       <c r="N663" t="inlineStr"/>
-      <c r="O663" t="inlineStr"/>
+      <c r="O663" t="inlineStr">
+        <is>
+          <t>L260201(대전 유성여고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="664">
       <c r="A664" t="n">
@@ -35380,7 +35944,11 @@
         </is>
       </c>
       <c r="N664" t="inlineStr"/>
-      <c r="O664" t="inlineStr"/>
+      <c r="O664" t="inlineStr">
+        <is>
+          <t>L240404(순천공고)-D</t>
+        </is>
+      </c>
     </row>
     <row r="665">
       <c r="A665" t="n">
@@ -35431,7 +35999,11 @@
         </is>
       </c>
       <c r="N665" t="inlineStr"/>
-      <c r="O665" t="inlineStr"/>
+      <c r="O665" t="inlineStr">
+        <is>
+          <t>L211201(대전 버드내중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="666">
       <c r="A666" t="n">
@@ -35482,7 +36054,11 @@
         </is>
       </c>
       <c r="N666" t="inlineStr"/>
-      <c r="O666" t="inlineStr"/>
+      <c r="O666" t="inlineStr">
+        <is>
+          <t>L230208(충남 청양중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="667">
       <c r="A667" t="n">
@@ -35533,7 +36109,11 @@
         </is>
       </c>
       <c r="N667" t="inlineStr"/>
-      <c r="O667" t="inlineStr"/>
+      <c r="O667" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="668">
       <c r="A668" t="n">
@@ -35584,7 +36164,11 @@
         </is>
       </c>
       <c r="N668" t="inlineStr"/>
-      <c r="O668" t="inlineStr"/>
+      <c r="O668" t="inlineStr">
+        <is>
+          <t>L240703(서산 음암중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" t="n">
@@ -35637,7 +36221,7 @@
       <c r="N669" t="inlineStr"/>
       <c r="O669" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>L241203(경주 선덕여중)-D</t>
         </is>
       </c>
     </row>
@@ -35690,7 +36274,11 @@
         </is>
       </c>
       <c r="N670" t="inlineStr"/>
-      <c r="O670" t="inlineStr"/>
+      <c r="O670" t="inlineStr">
+        <is>
+          <t>L260202(서산여고 2차증축)-A</t>
+        </is>
+      </c>
     </row>
     <row r="671">
       <c r="A671" t="n">
@@ -35741,7 +36329,11 @@
         </is>
       </c>
       <c r="N671" t="inlineStr"/>
-      <c r="O671" t="inlineStr"/>
+      <c r="O671" t="inlineStr">
+        <is>
+          <t>L230205(충남 태안중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="672">
       <c r="A672" t="n">
@@ -35792,7 +36384,11 @@
         </is>
       </c>
       <c r="N672" t="inlineStr"/>
-      <c r="O672" t="inlineStr"/>
+      <c r="O672" t="inlineStr">
+        <is>
+          <t>L241203(경주 선덕여중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="673">
       <c r="A673" t="n">
@@ -35900,7 +36496,7 @@
       <c r="N674" t="inlineStr"/>
       <c r="O674" t="inlineStr">
         <is>
-          <t>D250506(OSC 고도화 기술개발사업-PC공동주택)-E</t>
+          <t>M250902(BS3-25-A)-M</t>
         </is>
       </c>
     </row>
@@ -35953,7 +36549,11 @@
         </is>
       </c>
       <c r="N675" t="inlineStr"/>
-      <c r="O675" t="inlineStr"/>
+      <c r="O675" t="inlineStr">
+        <is>
+          <t>A251201(김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="676">
       <c r="A676" t="n">
@@ -36004,7 +36604,11 @@
         </is>
       </c>
       <c r="N676" t="inlineStr"/>
-      <c r="O676" t="inlineStr"/>
+      <c r="O676" t="inlineStr">
+        <is>
+          <t>L211201(대전 버드내중)-D</t>
+        </is>
+      </c>
     </row>
     <row r="677">
       <c r="A677" t="n">
@@ -36055,7 +36659,11 @@
         </is>
       </c>
       <c r="N677" t="inlineStr"/>
-      <c r="O677" t="inlineStr"/>
+      <c r="O677" t="inlineStr">
+        <is>
+          <t>L251005(홍성공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="678">
       <c r="A678" t="n">
@@ -36106,7 +36714,11 @@
         </is>
       </c>
       <c r="N678" t="inlineStr"/>
-      <c r="O678" t="inlineStr"/>
+      <c r="O678" t="inlineStr">
+        <is>
+          <t>L251203(위례푸른초)-A</t>
+        </is>
+      </c>
     </row>
     <row r="679">
       <c r="A679" t="n">
@@ -36157,7 +36769,11 @@
         </is>
       </c>
       <c r="N679" t="inlineStr"/>
-      <c r="O679" t="inlineStr"/>
+      <c r="O679" t="inlineStr">
+        <is>
+          <t>E221113(계산서취소분)-E</t>
+        </is>
+      </c>
     </row>
     <row r="680">
       <c r="A680" t="n">
@@ -36208,7 +36824,11 @@
         </is>
       </c>
       <c r="N680" t="inlineStr"/>
-      <c r="O680" t="inlineStr"/>
+      <c r="O680" t="inlineStr">
+        <is>
+          <t>I260103(대전 원신흥초)-E</t>
+        </is>
+      </c>
     </row>
     <row r="681">
       <c r="A681" t="n">
@@ -36369,7 +36989,11 @@
         </is>
       </c>
       <c r="N683" t="inlineStr"/>
-      <c r="O683" t="inlineStr"/>
+      <c r="O683" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="684">
       <c r="A684" t="n">
@@ -36475,7 +37099,11 @@
         </is>
       </c>
       <c r="N685" t="inlineStr"/>
-      <c r="O685" t="inlineStr"/>
+      <c r="O685" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="686">
       <c r="A686" t="n">
@@ -36583,7 +37211,7 @@
       <c r="N687" t="inlineStr"/>
       <c r="O687" t="inlineStr">
         <is>
-          <t>E250002(경비-공장)-E</t>
+          <t>A251201(김제공장)-E</t>
         </is>
       </c>
     </row>
@@ -36856,7 +37484,11 @@
         </is>
       </c>
       <c r="N692" t="inlineStr"/>
-      <c r="O692" t="inlineStr"/>
+      <c r="O692" t="inlineStr">
+        <is>
+          <t>I260101(일체형지붕-강내초,부곡초,조례초,연동초,청산고)-E</t>
+        </is>
+      </c>
     </row>
     <row r="693">
       <c r="A693" t="n">
@@ -36909,7 +37541,7 @@
       <c r="N693" t="inlineStr"/>
       <c r="O693" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4현장실)-C</t>
+          <t>L230208(충남 청양중)-D</t>
         </is>
       </c>
     </row>
@@ -36962,7 +37594,11 @@
         </is>
       </c>
       <c r="N694" t="inlineStr"/>
-      <c r="O694" t="inlineStr"/>
+      <c r="O694" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="695">
       <c r="A695" t="n">
@@ -37013,7 +37649,11 @@
         </is>
       </c>
       <c r="N695" t="inlineStr"/>
-      <c r="O695" t="inlineStr"/>
+      <c r="O695" t="inlineStr">
+        <is>
+          <t>M250902(BS3-25-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="696">
       <c r="A696" t="n">
@@ -37064,7 +37704,11 @@
         </is>
       </c>
       <c r="N696" t="inlineStr"/>
-      <c r="O696" t="inlineStr"/>
+      <c r="O696" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="697">
       <c r="A697" t="n">
@@ -37170,7 +37814,11 @@
         </is>
       </c>
       <c r="N698" t="inlineStr"/>
-      <c r="O698" t="inlineStr"/>
+      <c r="O698" t="inlineStr">
+        <is>
+          <t>I250416(야적장 갠트리크레인 설치공사)-C</t>
+        </is>
+      </c>
     </row>
     <row r="699">
       <c r="A699" t="n">
@@ -37221,7 +37869,11 @@
         </is>
       </c>
       <c r="N699" t="inlineStr"/>
-      <c r="O699" t="inlineStr"/>
+      <c r="O699" t="inlineStr">
+        <is>
+          <t>L251005(홍성공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="700">
       <c r="A700" t="n">
@@ -37327,7 +37979,11 @@
         </is>
       </c>
       <c r="N701" t="inlineStr"/>
-      <c r="O701" t="inlineStr"/>
+      <c r="O701" t="inlineStr">
+        <is>
+          <t>L241005(전주 우전초)-D</t>
+        </is>
+      </c>
     </row>
     <row r="702">
       <c r="A702" t="n">
@@ -37380,7 +38036,7 @@
       <c r="N702" t="inlineStr"/>
       <c r="O702" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4현장실)-C</t>
+          <t>E221113(계산서취소분)-E</t>
         </is>
       </c>
     </row>
@@ -37433,7 +38089,11 @@
         </is>
       </c>
       <c r="N703" t="inlineStr"/>
-      <c r="O703" t="inlineStr"/>
+      <c r="O703" t="inlineStr">
+        <is>
+          <t>S250401(대구 군위중)-A</t>
+        </is>
+      </c>
     </row>
     <row r="704">
       <c r="A704" t="n">
@@ -37486,7 +38146,7 @@
       <c r="N704" t="inlineStr"/>
       <c r="O704" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4현장실)-C</t>
+          <t>E221113(계산서취소분)-E</t>
         </is>
       </c>
     </row>
@@ -38309,7 +38969,11 @@
         </is>
       </c>
       <c r="N719" t="inlineStr"/>
-      <c r="O719" t="inlineStr"/>
+      <c r="O719" t="inlineStr">
+        <is>
+          <t>S250401(대구 군위중)-A</t>
+        </is>
+      </c>
     </row>
     <row r="720">
       <c r="A720" t="n">
@@ -38474,7 +39138,11 @@
         </is>
       </c>
       <c r="N722" t="inlineStr"/>
-      <c r="O722" t="inlineStr"/>
+      <c r="O722" t="inlineStr">
+        <is>
+          <t>L240404(순천공고)-D</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" t="n">
@@ -38580,7 +39248,11 @@
         </is>
       </c>
       <c r="N724" t="inlineStr"/>
-      <c r="O724" t="inlineStr"/>
+      <c r="O724" t="inlineStr">
+        <is>
+          <t>A251201(김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="725">
       <c r="A725" t="n">
@@ -38737,7 +39409,11 @@
         </is>
       </c>
       <c r="N727" t="inlineStr"/>
-      <c r="O727" t="inlineStr"/>
+      <c r="O727" t="inlineStr">
+        <is>
+          <t>L251005(홍성공고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="728">
       <c r="A728" t="n">
@@ -38788,7 +39464,11 @@
         </is>
       </c>
       <c r="N728" t="inlineStr"/>
-      <c r="O728" t="inlineStr"/>
+      <c r="O728" t="inlineStr">
+        <is>
+          <t>F250007(현장 하자/유지관리)-E</t>
+        </is>
+      </c>
     </row>
     <row r="729">
       <c r="A729" t="n">
@@ -38839,7 +39519,11 @@
         </is>
       </c>
       <c r="N729" t="inlineStr"/>
-      <c r="O729" t="inlineStr"/>
+      <c r="O729" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="730">
       <c r="A730" t="n">
@@ -38890,7 +39574,11 @@
         </is>
       </c>
       <c r="N730" t="inlineStr"/>
-      <c r="O730" t="inlineStr"/>
+      <c r="O730" t="inlineStr">
+        <is>
+          <t>A251201(김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="731">
       <c r="A731" t="n">
@@ -39047,7 +39735,11 @@
         </is>
       </c>
       <c r="N733" t="inlineStr"/>
-      <c r="O733" t="inlineStr"/>
+      <c r="O733" t="inlineStr">
+        <is>
+          <t>D250506(OSC 고도화 기술개발사업-PC공동주택)-E</t>
+        </is>
+      </c>
     </row>
     <row r="734">
       <c r="A734" t="n">
@@ -39153,7 +39845,11 @@
         </is>
       </c>
       <c r="N735" t="inlineStr"/>
-      <c r="O735" t="inlineStr"/>
+      <c r="O735" t="inlineStr">
+        <is>
+          <t>L260203(강원 양양고)-A</t>
+        </is>
+      </c>
     </row>
     <row r="736">
       <c r="A736" t="n">
@@ -39204,7 +39900,11 @@
         </is>
       </c>
       <c r="N736" t="inlineStr"/>
-      <c r="O736" t="inlineStr"/>
+      <c r="O736" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" t="n">
@@ -39255,7 +39955,11 @@
         </is>
       </c>
       <c r="N737" t="inlineStr"/>
-      <c r="O737" t="inlineStr"/>
+      <c r="O737" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="738">
       <c r="A738" t="n">
@@ -39365,7 +40069,11 @@
           <t>하자</t>
         </is>
       </c>
-      <c r="O739" t="inlineStr"/>
+      <c r="O739" t="inlineStr">
+        <is>
+          <t>L251202(청주성신학교)-A</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" t="n">
@@ -39416,7 +40124,11 @@
         </is>
       </c>
       <c r="N740" t="inlineStr"/>
-      <c r="O740" t="inlineStr"/>
+      <c r="O740" t="inlineStr">
+        <is>
+          <t>I260101(일체형지붕-강내초,부곡초,조례초,연동초,청산고)-E</t>
+        </is>
+      </c>
     </row>
     <row r="741">
       <c r="A741" t="n">
@@ -39750,7 +40462,11 @@
         </is>
       </c>
       <c r="N746" t="inlineStr"/>
-      <c r="O746" t="inlineStr"/>
+      <c r="O746" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="747">
       <c r="A747" t="n">
@@ -39801,7 +40517,11 @@
         </is>
       </c>
       <c r="N747" t="inlineStr"/>
-      <c r="O747" t="inlineStr"/>
+      <c r="O747" t="inlineStr">
+        <is>
+          <t>M260204(BS3-26-A)-M</t>
+        </is>
+      </c>
     </row>
     <row r="748">
       <c r="A748" t="n">
@@ -40107,7 +40827,11 @@
         </is>
       </c>
       <c r="N753" t="inlineStr"/>
-      <c r="O753" t="inlineStr"/>
+      <c r="O753" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="754">
       <c r="A754" t="n">
@@ -40158,7 +40882,11 @@
         </is>
       </c>
       <c r="N754" t="inlineStr"/>
-      <c r="O754" t="inlineStr"/>
+      <c r="O754" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="755">
       <c r="A755" t="n">
@@ -40209,7 +40937,11 @@
         </is>
       </c>
       <c r="N755" t="inlineStr"/>
-      <c r="O755" t="inlineStr"/>
+      <c r="O755" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="756">
       <c r="A756" t="n">
@@ -40364,7 +41096,7 @@
       <c r="N758" t="inlineStr"/>
       <c r="O758" t="inlineStr">
         <is>
-          <t>D250801(전북 혁신성장 R&amp;D+)-E</t>
+          <t>D221114(경상연구개발비)-E</t>
         </is>
       </c>
     </row>
@@ -40527,7 +41259,11 @@
         </is>
       </c>
       <c r="N761" t="inlineStr"/>
-      <c r="O761" t="inlineStr"/>
+      <c r="O761" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="762">
       <c r="A762" t="n">
@@ -40633,7 +41369,11 @@
         </is>
       </c>
       <c r="N763" t="inlineStr"/>
-      <c r="O763" t="inlineStr"/>
+      <c r="O763" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="764">
       <c r="A764" t="n">
@@ -40739,7 +41479,11 @@
         </is>
       </c>
       <c r="N765" t="inlineStr"/>
-      <c r="O765" t="inlineStr"/>
+      <c r="O765" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="766">
       <c r="A766" t="n">
@@ -40900,7 +41644,11 @@
         </is>
       </c>
       <c r="N768" t="inlineStr"/>
-      <c r="O768" t="inlineStr"/>
+      <c r="O768" t="inlineStr">
+        <is>
+          <t>E260002(경비-김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="769">
       <c r="A769" t="n">
@@ -40951,7 +41699,11 @@
         </is>
       </c>
       <c r="N769" t="inlineStr"/>
-      <c r="O769" t="inlineStr"/>
+      <c r="O769" t="inlineStr">
+        <is>
+          <t>E260002(경비-김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="770">
       <c r="A770" t="n">
@@ -41057,7 +41809,11 @@
         </is>
       </c>
       <c r="N771" t="inlineStr"/>
-      <c r="O771" t="inlineStr"/>
+      <c r="O771" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="772">
       <c r="A772" t="n">
@@ -41218,7 +41974,11 @@
         </is>
       </c>
       <c r="N774" t="inlineStr"/>
-      <c r="O774" t="inlineStr"/>
+      <c r="O774" t="inlineStr">
+        <is>
+          <t>E260002(경비-김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="775">
       <c r="A775" t="n">
@@ -41269,7 +42029,11 @@
         </is>
       </c>
       <c r="N775" t="inlineStr"/>
-      <c r="O775" t="inlineStr"/>
+      <c r="O775" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="776">
       <c r="A776" t="n">
@@ -41320,7 +42084,11 @@
         </is>
       </c>
       <c r="N776" t="inlineStr"/>
-      <c r="O776" t="inlineStr"/>
+      <c r="O776" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="777">
       <c r="A777" t="n">
@@ -41371,7 +42139,11 @@
         </is>
       </c>
       <c r="N777" t="inlineStr"/>
-      <c r="O777" t="inlineStr"/>
+      <c r="O777" t="inlineStr">
+        <is>
+          <t>A251201(김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="778">
       <c r="A778" t="n">
@@ -41422,7 +42194,11 @@
         </is>
       </c>
       <c r="N778" t="inlineStr"/>
-      <c r="O778" t="inlineStr"/>
+      <c r="O778" t="inlineStr">
+        <is>
+          <t>A251201(김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="779">
       <c r="A779" t="n">
@@ -41473,7 +42249,11 @@
         </is>
       </c>
       <c r="N779" t="inlineStr"/>
-      <c r="O779" t="inlineStr"/>
+      <c r="O779" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="780">
       <c r="A780" t="n">
@@ -41524,7 +42304,11 @@
         </is>
       </c>
       <c r="N780" t="inlineStr"/>
-      <c r="O780" t="inlineStr"/>
+      <c r="O780" t="inlineStr">
+        <is>
+          <t>E260002(경비-김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="781">
       <c r="A781" t="n">
@@ -41575,7 +42359,11 @@
         </is>
       </c>
       <c r="N781" t="inlineStr"/>
-      <c r="O781" t="inlineStr"/>
+      <c r="O781" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="782">
       <c r="A782" t="n">
@@ -41626,7 +42414,11 @@
         </is>
       </c>
       <c r="N782" t="inlineStr"/>
-      <c r="O782" t="inlineStr"/>
+      <c r="O782" t="inlineStr">
+        <is>
+          <t>E260002(경비-김제공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="783">
       <c r="A783" t="n">
@@ -41677,7 +42469,11 @@
         </is>
       </c>
       <c r="N783" t="inlineStr"/>
-      <c r="O783" t="inlineStr"/>
+      <c r="O783" t="inlineStr">
+        <is>
+          <t>E250001(경비-서울)-E</t>
+        </is>
+      </c>
     </row>
     <row r="784">
       <c r="A784" t="n">
@@ -41728,7 +42524,11 @@
         </is>
       </c>
       <c r="N784" t="inlineStr"/>
-      <c r="O784" t="inlineStr"/>
+      <c r="O784" t="inlineStr">
+        <is>
+          <t>F250007(현장 하자/유지관리)-E</t>
+        </is>
+      </c>
     </row>
     <row r="785">
       <c r="A785" t="n">
@@ -41779,7 +42579,11 @@
         </is>
       </c>
       <c r="N785" t="inlineStr"/>
-      <c r="O785" t="inlineStr"/>
+      <c r="O785" t="inlineStr">
+        <is>
+          <t>E250002(경비-공장)-E</t>
+        </is>
+      </c>
     </row>
     <row r="786">
       <c r="A786" t="n">
@@ -41832,7 +42636,7 @@
       <c r="N786" t="inlineStr"/>
       <c r="O786" t="inlineStr">
         <is>
-          <t>C240801(의왕초평A-4현장실)-C</t>
+          <t>E260002(경비-김제공장)-E</t>
         </is>
       </c>
     </row>
@@ -41885,7 +42689,11 @@
         </is>
       </c>
       <c r="N787" t="inlineStr"/>
-      <c r="O787" t="inlineStr"/>
+      <c r="O787" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="788">
       <c r="A788" t="n">
@@ -42046,7 +42854,11 @@
         </is>
       </c>
       <c r="N790" t="inlineStr"/>
-      <c r="O790" t="inlineStr"/>
+      <c r="O790" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="791">
       <c r="A791" t="n">
@@ -42097,7 +42909,11 @@
         </is>
       </c>
       <c r="N791" t="inlineStr"/>
-      <c r="O791" t="inlineStr"/>
+      <c r="O791" t="inlineStr">
+        <is>
+          <t>C240801(의왕초평A-4BL)-M</t>
+        </is>
+      </c>
     </row>
     <row r="792">
       <c r="A792" t="n">

</xml_diff>